<commit_message>
Cases and Checklist added
</commit_message>
<xml_diff>
--- a/Check.xlsx
+++ b/Check.xlsx
@@ -11,12 +11,27 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="73">
   <si>
-    <t>Авторизация</t>
+    <t>Экран загрузки</t>
   </si>
   <si>
     <t>Приоритет:</t>
+  </si>
+  <si>
+    <t>Проверить прогресс-бар на экране загрузки</t>
+  </si>
+  <si>
+    <t>Низкий</t>
+  </si>
+  <si>
+    <t>Проверить отображение изображения на экране загрузки</t>
+  </si>
+  <si>
+    <t>Проверить наличие цитаты на экране загрузки</t>
+  </si>
+  <si>
+    <t>Авторизация</t>
   </si>
   <si>
     <t>Проверить наличие полей для ввода логина и пароля</t>
@@ -43,16 +58,22 @@
     <t>Средний</t>
   </si>
   <si>
-    <t xml:space="preserve">Проверить автозаполнение логина/пароля (если предусмотрено) </t>
+    <t>Проверить повторный запуск приложения при выполненном входе</t>
   </si>
   <si>
-    <t>Низкий</t>
+    <t xml:space="preserve">Проверить автозаполнение логина/пароля (если предусмотрено) </t>
   </si>
   <si>
     <t>Главная страница</t>
   </si>
   <si>
-    <t xml:space="preserve">Проверить наличие блока новостей </t>
+    <t xml:space="preserve">Проверить наличие окна "News" </t>
+  </si>
+  <si>
+    <t>Проверить наличие стрелочки в окне "News"</t>
+  </si>
+  <si>
+    <t>Проверить кликабельность стрелочки в окне "News"</t>
   </si>
   <si>
     <t>Проверить наличие кнопки “ALL NEWS”</t>
@@ -80,7 +101,7 @@
     <t xml:space="preserve">Проверить корректную работу фильтра </t>
   </si>
   <si>
-    <t xml:space="preserve">Проверить фильтрацию по алфавиту </t>
+    <t>Проверить фильтрацию по дате добавления</t>
   </si>
   <si>
     <t xml:space="preserve">Проверить отображение пустого списка новостей </t>
@@ -104,7 +125,7 @@
     <t>Страница "Love is all"</t>
   </si>
   <si>
-    <t xml:space="preserve">Проверить переход на страницу "Love is all" с Главной страницы </t>
+    <t>Проверить переход на страницу "Love is all" с Главной страницы (иконка бабочки)</t>
   </si>
   <si>
     <t xml:space="preserve">Проверить отображение списка цитат </t>
@@ -164,7 +185,7 @@
     <t>Выход из аккаунта</t>
   </si>
   <si>
-    <t xml:space="preserve">Проверить наличие иконки аккаунта для выхода </t>
+    <t>Проверить наличие иконки аккаунта для выхода (иконка человечка)</t>
   </si>
   <si>
     <t xml:space="preserve">Проверить нажатие на иконку </t>
@@ -227,6 +248,7 @@
       <sz val="12.0"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <color theme="1"/>
@@ -241,7 +263,6 @@
       <sz val="12.0"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
     <font/>
     <font>
@@ -282,6 +303,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF00FF00"/>
+        <bgColor rgb="FF00FF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
         <bgColor rgb="FFFF0000"/>
       </patternFill>
@@ -290,12 +317,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFF9900"/>
         <bgColor rgb="FFFF9900"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00FF00"/>
-        <bgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -311,6 +332,28 @@
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
@@ -334,28 +377,6 @@
         <color rgb="FF000000"/>
       </bottom>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
@@ -365,50 +386,50 @@
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+      <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="2" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="2" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="2" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="6" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="6" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -417,7 +438,7 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="3" fillId="7" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="7" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -695,7 +716,7 @@
       <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="3"/>
@@ -722,7 +743,7 @@
       <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="3"/>
@@ -746,12 +767,10 @@
       <c r="U4" s="3"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>3</v>
-      </c>
+      <c r="B5" s="7"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
@@ -773,11 +792,11 @@
       <c r="U5" s="3"/>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>3</v>
+      <c r="B6" s="9" t="s">
+        <v>8</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
@@ -800,11 +819,11 @@
       <c r="U6" s="3"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>8</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>9</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
@@ -827,11 +846,11 @@
       <c r="U7" s="3"/>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="8" t="s">
-        <v>11</v>
+      <c r="B8" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
@@ -854,10 +873,12 @@
       <c r="U8" s="3"/>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="s">
-        <v>12</v>
+      <c r="A9" s="8" t="s">
+        <v>11</v>
       </c>
-      <c r="B9" s="10"/>
+      <c r="B9" s="10" t="s">
+        <v>8</v>
+      </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -879,11 +900,11 @@
       <c r="U9" s="3"/>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="s">
-        <v>13</v>
+      <c r="A10" s="8" t="s">
+        <v>12</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>3</v>
+      <c r="B10" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
@@ -906,11 +927,11 @@
       <c r="U10" s="3"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="11" t="s">
         <v>14</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>3</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
@@ -933,11 +954,11 @@
       <c r="U11" s="3"/>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="6" t="s">
-        <v>3</v>
+      <c r="B12" s="11" t="s">
+        <v>14</v>
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
@@ -960,10 +981,12 @@
       <c r="U12" s="3"/>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="10"/>
+      <c r="B13" s="5" t="s">
+        <v>3</v>
+      </c>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
@@ -985,12 +1008,10 @@
       <c r="U13" s="3"/>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="6" t="s">
-        <v>3</v>
-      </c>
+      <c r="B14" s="13"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
@@ -1012,11 +1033,11 @@
       <c r="U14" s="3"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="6" t="s">
-        <v>3</v>
+      <c r="B15" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
@@ -1039,11 +1060,11 @@
       <c r="U15" s="3"/>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="6" t="s">
-        <v>3</v>
+      <c r="B16" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
@@ -1066,11 +1087,11 @@
       <c r="U16" s="3"/>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="6" t="s">
-        <v>3</v>
+      <c r="B17" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
@@ -1093,11 +1114,11 @@
       <c r="U17" s="3"/>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="7" t="s">
-        <v>9</v>
+      <c r="B18" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
@@ -1120,11 +1141,11 @@
       <c r="U18" s="3"/>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="7" t="s">
-        <v>9</v>
+      <c r="B19" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
@@ -1146,13 +1167,11 @@
       <c r="T19" s="3"/>
       <c r="U19" s="3"/>
     </row>
-    <row r="20">
-      <c r="A20" s="11" t="s">
+    <row r="20" ht="18.75" customHeight="1">
+      <c r="A20" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="8" t="s">
-        <v>11</v>
-      </c>
+      <c r="B20" s="13"/>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
@@ -1174,10 +1193,12 @@
       <c r="U20" s="3"/>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="13"/>
+      <c r="B21" s="10" t="s">
+        <v>8</v>
+      </c>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
@@ -1202,8 +1223,8 @@
       <c r="A22" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B22" s="7" t="s">
-        <v>9</v>
+      <c r="B22" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
@@ -1229,8 +1250,8 @@
       <c r="A23" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="7" t="s">
-        <v>9</v>
+      <c r="B23" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
@@ -1256,8 +1277,8 @@
       <c r="A24" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B24" s="7" t="s">
-        <v>9</v>
+      <c r="B24" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
@@ -1280,11 +1301,11 @@
       <c r="U24" s="3"/>
     </row>
     <row r="25">
-      <c r="A25" s="14" t="s">
+      <c r="A25" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="6" t="s">
-        <v>3</v>
+      <c r="B25" s="11" t="s">
+        <v>14</v>
       </c>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
@@ -1307,10 +1328,12 @@
       <c r="U25" s="3"/>
     </row>
     <row r="26">
-      <c r="A26" s="15" t="s">
+      <c r="A26" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B26" s="13"/>
+      <c r="B26" s="11" t="s">
+        <v>14</v>
+      </c>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
@@ -1332,10 +1355,10 @@
       <c r="U26" s="3"/>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="s">
+      <c r="A27" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="5" t="s">
         <v>3</v>
       </c>
       <c r="C27" s="3"/>
@@ -1359,12 +1382,10 @@
       <c r="U27" s="3"/>
     </row>
     <row r="28">
-      <c r="A28" s="11" t="s">
+      <c r="A28" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="B28" s="6" t="s">
-        <v>3</v>
-      </c>
+      <c r="B28" s="7"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
@@ -1386,11 +1407,11 @@
       <c r="U28" s="3"/>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="s">
+      <c r="A29" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B29" s="7" t="s">
-        <v>9</v>
+      <c r="B29" s="11" t="s">
+        <v>14</v>
       </c>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
@@ -1413,11 +1434,11 @@
       <c r="U29" s="3"/>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="s">
+      <c r="A30" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="B30" s="7" t="s">
-        <v>9</v>
+      <c r="B30" s="11" t="s">
+        <v>14</v>
       </c>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
@@ -1440,10 +1461,12 @@
       <c r="U30" s="3"/>
     </row>
     <row r="31">
-      <c r="A31" s="16" t="s">
+      <c r="A31" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B31" s="13"/>
+      <c r="B31" s="11" t="s">
+        <v>14</v>
+      </c>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
@@ -1465,11 +1488,11 @@
       <c r="U31" s="3"/>
     </row>
     <row r="32">
-      <c r="A32" s="11" t="s">
+      <c r="A32" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="B32" s="6" t="s">
-        <v>3</v>
+      <c r="B32" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
@@ -1492,12 +1515,10 @@
       <c r="U32" s="3"/>
     </row>
     <row r="33">
-      <c r="A33" s="11" t="s">
+      <c r="A33" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B33" s="6" t="s">
-        <v>3</v>
-      </c>
+      <c r="B33" s="7"/>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
@@ -1519,11 +1540,11 @@
       <c r="U33" s="3"/>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="s">
+      <c r="A34" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B34" s="6" t="s">
-        <v>3</v>
+      <c r="B34" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
@@ -1546,11 +1567,11 @@
       <c r="U34" s="3"/>
     </row>
     <row r="35">
-      <c r="A35" s="11" t="s">
+      <c r="A35" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="6" t="s">
-        <v>3</v>
+      <c r="B35" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
@@ -1573,11 +1594,11 @@
       <c r="U35" s="3"/>
     </row>
     <row r="36">
-      <c r="A36" s="11" t="s">
+      <c r="A36" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B36" s="7" t="s">
-        <v>9</v>
+      <c r="B36" s="11" t="s">
+        <v>14</v>
       </c>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
@@ -1600,10 +1621,12 @@
       <c r="U36" s="3"/>
     </row>
     <row r="37">
-      <c r="A37" s="17" t="s">
+      <c r="A37" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B37" s="13"/>
+      <c r="B37" s="11" t="s">
+        <v>14</v>
+      </c>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
@@ -1625,12 +1648,10 @@
       <c r="U37" s="3"/>
     </row>
     <row r="38">
-      <c r="A38" s="11" t="s">
+      <c r="A38" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="B38" s="6" t="s">
-        <v>3</v>
-      </c>
+      <c r="B38" s="7"/>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
@@ -1652,11 +1673,11 @@
       <c r="U38" s="3"/>
     </row>
     <row r="39">
-      <c r="A39" s="11" t="s">
+      <c r="A39" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B39" s="6" t="s">
-        <v>3</v>
+      <c r="B39" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
@@ -1679,11 +1700,11 @@
       <c r="U39" s="3"/>
     </row>
     <row r="40">
-      <c r="A40" s="11" t="s">
+      <c r="A40" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B40" s="6" t="s">
-        <v>3</v>
+      <c r="B40" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
@@ -1706,11 +1727,11 @@
       <c r="U40" s="3"/>
     </row>
     <row r="41">
-      <c r="A41" s="11" t="s">
+      <c r="A41" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B41" s="6" t="s">
-        <v>3</v>
+      <c r="B41" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
@@ -1733,11 +1754,11 @@
       <c r="U41" s="3"/>
     </row>
     <row r="42">
-      <c r="A42" s="18" t="s">
+      <c r="A42" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B42" s="6" t="s">
-        <v>3</v>
+      <c r="B42" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C42" s="3"/>
       <c r="D42" s="3"/>
@@ -1760,11 +1781,11 @@
       <c r="U42" s="3"/>
     </row>
     <row r="43">
-      <c r="A43" s="11" t="s">
+      <c r="A43" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B43" s="7" t="s">
-        <v>9</v>
+      <c r="B43" s="11" t="s">
+        <v>14</v>
       </c>
       <c r="C43" s="3"/>
       <c r="D43" s="3"/>
@@ -1787,12 +1808,10 @@
       <c r="U43" s="3"/>
     </row>
     <row r="44">
-      <c r="A44" s="11" t="s">
+      <c r="A44" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="B44" s="7" t="s">
-        <v>9</v>
-      </c>
+      <c r="B44" s="7"/>
       <c r="C44" s="3"/>
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
@@ -1814,11 +1833,11 @@
       <c r="U44" s="3"/>
     </row>
     <row r="45">
-      <c r="A45" s="11" t="s">
+      <c r="A45" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B45" s="7" t="s">
-        <v>9</v>
+      <c r="B45" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C45" s="3"/>
       <c r="D45" s="3"/>
@@ -1841,10 +1860,12 @@
       <c r="U45" s="3"/>
     </row>
     <row r="46">
-      <c r="A46" s="9" t="s">
+      <c r="A46" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B46" s="10"/>
+      <c r="B46" s="10" t="s">
+        <v>8</v>
+      </c>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
       <c r="E46" s="3"/>
@@ -1866,11 +1887,11 @@
       <c r="U46" s="3"/>
     </row>
     <row r="47">
-      <c r="A47" s="19" t="s">
+      <c r="A47" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B47" s="6" t="s">
-        <v>3</v>
+      <c r="B47" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
@@ -1893,11 +1914,11 @@
       <c r="U47" s="3"/>
     </row>
     <row r="48">
-      <c r="A48" s="19" t="s">
+      <c r="A48" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B48" s="6" t="s">
-        <v>3</v>
+      <c r="B48" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C48" s="3"/>
       <c r="D48" s="3"/>
@@ -1920,11 +1941,11 @@
       <c r="U48" s="3"/>
     </row>
     <row r="49">
-      <c r="A49" s="19" t="s">
+      <c r="A49" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="B49" s="6" t="s">
-        <v>3</v>
+      <c r="B49" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C49" s="3"/>
       <c r="D49" s="3"/>
@@ -1947,11 +1968,11 @@
       <c r="U49" s="3"/>
     </row>
     <row r="50">
-      <c r="A50" s="19" t="s">
+      <c r="A50" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B50" s="7" t="s">
-        <v>9</v>
+      <c r="B50" s="11" t="s">
+        <v>14</v>
       </c>
       <c r="C50" s="3"/>
       <c r="D50" s="3"/>
@@ -1974,10 +1995,12 @@
       <c r="U50" s="3"/>
     </row>
     <row r="51">
-      <c r="A51" s="9" t="s">
+      <c r="A51" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B51" s="10"/>
+      <c r="B51" s="11" t="s">
+        <v>14</v>
+      </c>
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>
@@ -1999,11 +2022,11 @@
       <c r="U51" s="3"/>
     </row>
     <row r="52">
-      <c r="A52" s="20" t="s">
+      <c r="A52" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B52" s="6" t="s">
-        <v>3</v>
+      <c r="B52" s="11" t="s">
+        <v>14</v>
       </c>
       <c r="C52" s="3"/>
       <c r="D52" s="3"/>
@@ -2026,12 +2049,10 @@
       <c r="U52" s="3"/>
     </row>
     <row r="53">
-      <c r="A53" s="20" t="s">
+      <c r="A53" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="B53" s="6" t="s">
-        <v>3</v>
-      </c>
+      <c r="B53" s="13"/>
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
       <c r="E53" s="3"/>
@@ -2053,11 +2074,11 @@
       <c r="U53" s="3"/>
     </row>
     <row r="54">
-      <c r="A54" s="20" t="s">
+      <c r="A54" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="B54" s="6" t="s">
-        <v>3</v>
+      <c r="B54" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C54" s="3"/>
       <c r="D54" s="3"/>
@@ -2080,11 +2101,11 @@
       <c r="U54" s="3"/>
     </row>
     <row r="55">
-      <c r="A55" s="20" t="s">
+      <c r="A55" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="B55" s="6" t="s">
-        <v>3</v>
+      <c r="B55" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C55" s="3"/>
       <c r="D55" s="3"/>
@@ -2107,11 +2128,11 @@
       <c r="U55" s="3"/>
     </row>
     <row r="56">
-      <c r="A56" s="20" t="s">
+      <c r="A56" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="B56" s="6" t="s">
-        <v>3</v>
+      <c r="B56" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C56" s="3"/>
       <c r="D56" s="3"/>
@@ -2134,10 +2155,12 @@
       <c r="U56" s="3"/>
     </row>
     <row r="57">
-      <c r="A57" s="15" t="s">
+      <c r="A57" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="B57" s="13"/>
+      <c r="B57" s="11" t="s">
+        <v>14</v>
+      </c>
       <c r="C57" s="3"/>
       <c r="D57" s="3"/>
       <c r="E57" s="3"/>
@@ -2159,12 +2182,10 @@
       <c r="U57" s="3"/>
     </row>
     <row r="58">
-      <c r="A58" s="11" t="s">
+      <c r="A58" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B58" s="6" t="s">
-        <v>3</v>
-      </c>
+      <c r="B58" s="13"/>
       <c r="C58" s="3"/>
       <c r="D58" s="3"/>
       <c r="E58" s="3"/>
@@ -2186,11 +2207,11 @@
       <c r="U58" s="3"/>
     </row>
     <row r="59">
-      <c r="A59" s="11" t="s">
+      <c r="A59" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="B59" s="7" t="s">
-        <v>9</v>
+      <c r="B59" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C59" s="3"/>
       <c r="D59" s="3"/>
@@ -2213,11 +2234,11 @@
       <c r="U59" s="3"/>
     </row>
     <row r="60">
-      <c r="A60" s="11" t="s">
+      <c r="A60" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="B60" s="7" t="s">
-        <v>9</v>
+      <c r="B60" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C60" s="3"/>
       <c r="D60" s="3"/>
@@ -2240,11 +2261,11 @@
       <c r="U60" s="3"/>
     </row>
     <row r="61">
-      <c r="A61" s="11" t="s">
+      <c r="A61" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="B61" s="7" t="s">
-        <v>9</v>
+      <c r="B61" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C61" s="3"/>
       <c r="D61" s="3"/>
@@ -2267,11 +2288,11 @@
       <c r="U61" s="3"/>
     </row>
     <row r="62">
-      <c r="A62" s="11" t="s">
+      <c r="A62" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="B62" s="7" t="s">
-        <v>9</v>
+      <c r="B62" s="10" t="s">
+        <v>8</v>
       </c>
       <c r="C62" s="3"/>
       <c r="D62" s="3"/>
@@ -2294,8 +2315,12 @@
       <c r="U62" s="3"/>
     </row>
     <row r="63">
-      <c r="A63" s="3"/>
-      <c r="B63" s="3"/>
+      <c r="A63" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="B63" s="10" t="s">
+        <v>8</v>
+      </c>
       <c r="C63" s="3"/>
       <c r="D63" s="3"/>
       <c r="E63" s="3"/>
@@ -2317,8 +2342,10 @@
       <c r="U63" s="3"/>
     </row>
     <row r="64">
-      <c r="A64" s="3"/>
-      <c r="B64" s="3"/>
+      <c r="A64" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B64" s="7"/>
       <c r="C64" s="3"/>
       <c r="D64" s="3"/>
       <c r="E64" s="3"/>
@@ -2340,8 +2367,12 @@
       <c r="U64" s="3"/>
     </row>
     <row r="65">
-      <c r="A65" s="3"/>
-      <c r="B65" s="3"/>
+      <c r="A65" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B65" s="10" t="s">
+        <v>8</v>
+      </c>
       <c r="C65" s="3"/>
       <c r="D65" s="3"/>
       <c r="E65" s="3"/>
@@ -2363,8 +2394,12 @@
       <c r="U65" s="3"/>
     </row>
     <row r="66">
-      <c r="A66" s="3"/>
-      <c r="B66" s="3"/>
+      <c r="A66" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B66" s="11" t="s">
+        <v>14</v>
+      </c>
       <c r="C66" s="3"/>
       <c r="D66" s="3"/>
       <c r="E66" s="3"/>
@@ -2386,8 +2421,12 @@
       <c r="U66" s="3"/>
     </row>
     <row r="67">
-      <c r="A67" s="3"/>
-      <c r="B67" s="3"/>
+      <c r="A67" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B67" s="11" t="s">
+        <v>14</v>
+      </c>
       <c r="C67" s="3"/>
       <c r="D67" s="3"/>
       <c r="E67" s="3"/>
@@ -2409,8 +2448,12 @@
       <c r="U67" s="3"/>
     </row>
     <row r="68">
-      <c r="A68" s="3"/>
-      <c r="B68" s="3"/>
+      <c r="A68" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B68" s="11" t="s">
+        <v>14</v>
+      </c>
       <c r="C68" s="3"/>
       <c r="D68" s="3"/>
       <c r="E68" s="3"/>
@@ -2432,8 +2475,12 @@
       <c r="U68" s="3"/>
     </row>
     <row r="69">
-      <c r="A69" s="3"/>
-      <c r="B69" s="3"/>
+      <c r="A69" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B69" s="11" t="s">
+        <v>14</v>
+      </c>
       <c r="C69" s="3"/>
       <c r="D69" s="3"/>
       <c r="E69" s="3"/>
@@ -18669,20 +18716,44 @@
       <c r="T774" s="3"/>
       <c r="U774" s="3"/>
     </row>
+    <row r="775">
+      <c r="A775" s="3"/>
+      <c r="B775" s="3"/>
+      <c r="C775" s="3"/>
+      <c r="D775" s="3"/>
+      <c r="E775" s="3"/>
+      <c r="F775" s="3"/>
+      <c r="G775" s="3"/>
+      <c r="H775" s="3"/>
+      <c r="I775" s="3"/>
+      <c r="J775" s="3"/>
+      <c r="K775" s="3"/>
+      <c r="L775" s="3"/>
+      <c r="M775" s="3"/>
+      <c r="N775" s="3"/>
+      <c r="O775" s="3"/>
+      <c r="P775" s="3"/>
+      <c r="Q775" s="3"/>
+      <c r="R775" s="3"/>
+      <c r="S775" s="3"/>
+      <c r="T775" s="3"/>
+      <c r="U775" s="3"/>
+    </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="A51:B51"/>
-    <mergeCell ref="A57:B57"/>
+  <mergeCells count="10">
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="A58:B58"/>
+    <mergeCell ref="A64:B64"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A44:B44"/>
   </mergeCells>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="B2:B8 B10:B12 B14:B20 B22:B25 B27:B30 B32:B36 B38:B45 B47:B50 B52:B56 B58:B62">
+    <dataValidation type="list" allowBlank="1" sqref="B2:B4 B6:B13 B15:B19 B21:B27 B29:B32 B34:B37 B39:B43 B45:B52 B54:B57 B59:B63 B65:B69">
       <formula1>"Высокий,Средний,Низкий"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>